<commit_message>
Wolfssl manual inspection done
</commit_message>
<xml_diff>
--- a/ExcelFiles/WolfSSL_Select.xlsx
+++ b/ExcelFiles/WolfSSL_Select.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muyeedahmed/Desktop/Gitcode/LLMVerification/ExcelFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E92388D8-FCFB-9A46-BB51-0EBCAF7ABCD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E55A518A-44BE-B049-B883-61DB3256096D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1320" yWindow="500" windowWidth="27480" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="wolfssl" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">wolfssl!$A$1:$T$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">wolfssl!$A$1:$V$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="116">
   <si>
     <t>Version</t>
   </si>
@@ -363,6 +363,18 @@
   </si>
   <si>
     <t>Error: undeclared identifier</t>
+  </si>
+  <si>
+    <t>Ministral</t>
+  </si>
+  <si>
+    <t>Qwen3</t>
+  </si>
+  <si>
+    <t>No Change</t>
+  </si>
+  <si>
+    <t>Empty/Incomplete Files</t>
   </si>
 </sst>
 </file>
@@ -761,20 +773,23 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:U23"/>
+  <dimension ref="A1:W23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="9.1640625" customWidth="1"/>
-    <col min="2" max="2" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.5" customWidth="1"/>
-    <col min="6" max="6" width="14.33203125" customWidth="1"/>
-    <col min="7" max="7" width="8.83203125"/>
-    <col min="8" max="8" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3" customWidth="1"/>
+    <col min="2" max="2" width="3.83203125" customWidth="1"/>
+    <col min="3" max="3" width="3.1640625" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" customWidth="1"/>
+    <col min="5" max="5" width="1.6640625" customWidth="1"/>
+    <col min="6" max="6" width="2" customWidth="1"/>
+    <col min="7" max="7" width="14.1640625" customWidth="1"/>
+    <col min="8" max="8" width="3.83203125" customWidth="1"/>
+    <col min="9" max="9" width="2.5" customWidth="1"/>
     <col min="10" max="11" width="3.1640625" customWidth="1"/>
-    <col min="12" max="12" width="9.83203125" customWidth="1"/>
+    <col min="12" max="12" width="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="14" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:23" s="14" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -815,29 +830,35 @@
         <v>9</v>
       </c>
       <c r="N1" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="O1" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="P1" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="Q1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="P1" s="13" t="s">
+      <c r="R1" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="S1" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="T1" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="S1" s="8" t="s">
+      <c r="U1" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="V1" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="U1"/>
-    </row>
-    <row r="2" spans="1:21" ht="15" x14ac:dyDescent="0.2">
+      <c r="W1"/>
+    </row>
+    <row r="2" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>44</v>
       </c>
@@ -879,23 +900,25 @@
       </c>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
-      <c r="P2" s="6" t="s">
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="Q2">
-        <v>19939</v>
-      </c>
-      <c r="R2">
-        <v>20150</v>
       </c>
       <c r="S2">
         <v>19939</v>
       </c>
       <c r="T2">
+        <v>20150</v>
+      </c>
+      <c r="U2">
+        <v>19939</v>
+      </c>
+      <c r="V2">
         <v>20142</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>51</v>
       </c>
@@ -935,15 +958,17 @@
       <c r="M3" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="N3" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="N3" s="1"/>
       <c r="O3" s="1"/>
-      <c r="P3" s="6" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" ht="15" x14ac:dyDescent="0.2">
+      <c r="P3" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q3" s="1"/>
+      <c r="R3" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>51</v>
       </c>
@@ -983,21 +1008,23 @@
       <c r="M4" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="N4" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="N4" s="1"/>
       <c r="O4" s="1"/>
-      <c r="P4" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="S4">
+      <c r="P4" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q4" s="1"/>
+      <c r="R4" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="U4">
         <v>11864</v>
       </c>
-      <c r="T4">
+      <c r="V4">
         <v>12272</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>26</v>
       </c>
@@ -1038,14 +1065,20 @@
         <v>110</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="O5" s="1"/>
-      <c r="P5" s="6" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" ht="15" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q5" s="1"/>
+      <c r="R5" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>26</v>
       </c>
@@ -1085,27 +1118,29 @@
       <c r="M6" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="N6" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="N6" s="1"/>
       <c r="O6" s="1"/>
-      <c r="P6" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q6">
-        <v>8782</v>
-      </c>
-      <c r="R6">
-        <v>9606</v>
+      <c r="P6" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q6" s="1"/>
+      <c r="R6" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="S6">
         <v>8782</v>
       </c>
       <c r="T6">
+        <v>9606</v>
+      </c>
+      <c r="U6">
+        <v>8782</v>
+      </c>
+      <c r="V6">
         <v>9598</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -1146,20 +1181,26 @@
         <v>110</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="O7" s="1"/>
-      <c r="P7" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="S7">
+        <v>115</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q7" s="1"/>
+      <c r="R7" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="U7">
         <v>993</v>
       </c>
-      <c r="T7">
+      <c r="V7">
         <v>1156</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>12</v>
       </c>
@@ -1200,26 +1241,32 @@
         <v>110</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="O8" s="1"/>
-      <c r="P8" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q8">
+        <v>115</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q8" s="1"/>
+      <c r="R8" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="S8">
         <v>1692</v>
       </c>
-      <c r="R8">
+      <c r="T8">
         <v>1813</v>
       </c>
-      <c r="S8">
+      <c r="U8">
         <v>1797</v>
       </c>
-      <c r="T8">
+      <c r="V8">
         <v>1914</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
@@ -1259,27 +1306,29 @@
       <c r="M9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="N9" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="N9" s="1"/>
       <c r="O9" s="1"/>
-      <c r="P9" s="6" t="s">
+      <c r="P9" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q9" s="1"/>
+      <c r="R9" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="Q9">
+      <c r="S9">
         <v>2481</v>
       </c>
-      <c r="R9">
+      <c r="T9">
         <v>2660</v>
       </c>
-      <c r="S9">
+      <c r="U9">
         <v>2516</v>
       </c>
-      <c r="T9">
+      <c r="V9">
         <v>2695</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>26</v>
       </c>
@@ -1321,23 +1370,25 @@
       </c>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
-      <c r="P10" s="6" t="s">
+      <c r="P10" s="1"/>
+      <c r="Q10" s="1"/>
+      <c r="R10" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="Q10">
+      <c r="S10">
         <v>654</v>
       </c>
-      <c r="R10">
+      <c r="T10">
         <v>686</v>
       </c>
-      <c r="S10">
+      <c r="U10">
         <v>653</v>
       </c>
-      <c r="T10">
+      <c r="V10">
         <v>685</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>44</v>
       </c>
@@ -1378,17 +1429,17 @@
         <v>110</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="O11" s="1"/>
-      <c r="P11" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q11">
-        <v>346</v>
-      </c>
-      <c r="R11">
-        <v>583</v>
+        <v>115</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q11" s="1"/>
+      <c r="R11" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="S11">
         <v>346</v>
@@ -1396,8 +1447,14 @@
       <c r="T11">
         <v>583</v>
       </c>
-    </row>
-    <row r="12" spans="1:21" ht="15" x14ac:dyDescent="0.2">
+      <c r="U11">
+        <v>346</v>
+      </c>
+      <c r="V11">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>26</v>
       </c>
@@ -1431,15 +1488,21 @@
       <c r="M12" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="N12" s="1"/>
+      <c r="N12" s="1" t="s">
+        <v>115</v>
+      </c>
       <c r="O12" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="P12" s="1"/>
+      <c r="Q12" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="P12" s="6" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="13" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R12" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>40</v>
       </c>
@@ -1479,27 +1542,29 @@
       <c r="M13" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="N13" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="N13" s="1"/>
       <c r="O13" s="1"/>
-      <c r="P13" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q13">
+      <c r="P13" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q13" s="1"/>
+      <c r="R13" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="S13">
         <v>20913</v>
       </c>
-      <c r="R13">
+      <c r="T13">
         <v>21203</v>
       </c>
-      <c r="S13">
+      <c r="U13">
         <v>20905</v>
       </c>
-      <c r="T13">
+      <c r="V13">
         <v>21195</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>51</v>
       </c>
@@ -1539,27 +1604,29 @@
       <c r="M14" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="N14" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="N14" s="1"/>
       <c r="O14" s="1"/>
-      <c r="P14" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q14">
-        <v>1030</v>
-      </c>
-      <c r="R14">
-        <v>1187</v>
+      <c r="P14" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q14" s="1"/>
+      <c r="R14" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="S14">
         <v>1030</v>
       </c>
       <c r="T14">
+        <v>1187</v>
+      </c>
+      <c r="U14">
+        <v>1030</v>
+      </c>
+      <c r="V14">
         <v>1184</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>26</v>
       </c>
@@ -1601,23 +1668,25 @@
       </c>
       <c r="N15" s="1"/>
       <c r="O15" s="1"/>
-      <c r="P15" s="6" t="s">
+      <c r="P15" s="1"/>
+      <c r="Q15" s="1"/>
+      <c r="R15" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="Q15">
-        <v>12845</v>
-      </c>
-      <c r="R15">
-        <v>13109</v>
       </c>
       <c r="S15">
         <v>12845</v>
       </c>
       <c r="T15">
+        <v>13109</v>
+      </c>
+      <c r="U15">
+        <v>12845</v>
+      </c>
+      <c r="V15">
         <v>13253</v>
       </c>
     </row>
-    <row r="16" spans="1:21" ht="15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>12</v>
       </c>
@@ -1658,20 +1727,26 @@
         <v>110</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="O16" s="1"/>
-      <c r="P16" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="S16">
+        <v>115</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="P16" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q16" s="1"/>
+      <c r="R16" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="U16">
         <v>1</v>
       </c>
-      <c r="T16">
+      <c r="V16">
         <v>164</v>
       </c>
     </row>
-    <row r="17" spans="1:20" ht="15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>51</v>
       </c>
@@ -1711,18 +1786,14 @@
       <c r="M17" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="N17" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="N17" s="1"/>
       <c r="O17" s="1"/>
-      <c r="P17" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q17">
-        <v>14423</v>
-      </c>
-      <c r="R17">
-        <v>14564</v>
+      <c r="P17" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q17" s="1"/>
+      <c r="R17" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="S17">
         <v>14423</v>
@@ -1730,8 +1801,14 @@
       <c r="T17">
         <v>14564</v>
       </c>
-    </row>
-    <row r="18" spans="1:20" ht="15" x14ac:dyDescent="0.2">
+      <c r="U17">
+        <v>14423</v>
+      </c>
+      <c r="V17">
+        <v>14564</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>26</v>
       </c>
@@ -1771,27 +1848,29 @@
       <c r="M18" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="N18" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="N18" s="1"/>
       <c r="O18" s="1"/>
-      <c r="P18" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q18">
+      <c r="P18" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q18" s="1"/>
+      <c r="R18" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="S18">
         <v>38033</v>
       </c>
-      <c r="R18">
+      <c r="T18">
         <v>38113</v>
       </c>
-      <c r="S18">
+      <c r="U18">
         <v>38034</v>
       </c>
-      <c r="T18">
+      <c r="V18">
         <v>38111</v>
       </c>
     </row>
-    <row r="19" spans="1:20" ht="15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>40</v>
       </c>
@@ -1826,14 +1905,20 @@
         <v>110</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="O19" s="1"/>
-      <c r="P19" s="6" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20" ht="15" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="P19" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q19" s="1"/>
+      <c r="R19" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>44</v>
       </c>
@@ -1873,27 +1958,29 @@
       <c r="M20" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="N20" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="N20" s="1"/>
       <c r="O20" s="1"/>
-      <c r="P20" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q20">
+      <c r="P20" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q20" s="1"/>
+      <c r="R20" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="S20">
         <v>6437</v>
       </c>
-      <c r="R20">
+      <c r="T20">
         <v>6504</v>
       </c>
-      <c r="S20">
+      <c r="U20">
         <v>6443</v>
       </c>
-      <c r="T20">
+      <c r="V20">
         <v>6513</v>
       </c>
     </row>
-    <row r="21" spans="1:20" ht="15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>26</v>
       </c>
@@ -1935,23 +2022,25 @@
       </c>
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
-      <c r="P21" s="6" t="s">
+      <c r="P21" s="1"/>
+      <c r="Q21" s="1"/>
+      <c r="R21" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="Q21">
+      <c r="S21">
         <v>20966</v>
       </c>
-      <c r="R21">
+      <c r="T21">
         <v>21004</v>
       </c>
-      <c r="S21">
+      <c r="U21">
         <v>20965</v>
       </c>
-      <c r="T21">
+      <c r="V21">
         <v>21003</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>12</v>
       </c>
@@ -1992,26 +2081,32 @@
         <v>109</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="O22" s="1"/>
-      <c r="P22" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q22">
+        <v>114</v>
+      </c>
+      <c r="O22" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="P22" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q22" s="1"/>
+      <c r="R22" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="S22">
         <v>6</v>
       </c>
-      <c r="R22">
+      <c r="T22">
         <v>119</v>
       </c>
-      <c r="S22">
+      <c r="U22">
         <v>69</v>
       </c>
-      <c r="T22">
+      <c r="V22">
         <v>185</v>
       </c>
     </row>
-    <row r="23" spans="1:20" ht="15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>12</v>
       </c>
@@ -2052,27 +2147,33 @@
         <v>110</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="O23" s="1"/>
-      <c r="P23" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q23">
+        <v>110</v>
+      </c>
+      <c r="O23" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="P23" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q23" s="1"/>
+      <c r="R23" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="S23">
         <v>325</v>
       </c>
-      <c r="R23">
+      <c r="T23">
         <v>419</v>
       </c>
-      <c r="S23">
+      <c r="U23">
         <v>323</v>
       </c>
-      <c r="T23">
+      <c r="V23">
         <v>417</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:V1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>

<commit_message>
RunClang: wolfssl done manually
</commit_message>
<xml_diff>
--- a/ExcelFiles/WolfSSL_Select.xlsx
+++ b/ExcelFiles/WolfSSL_Select.xlsx
@@ -8,22 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muyeedahmed/Desktop/Gitcode/LLMVerification/ExcelFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E55A518A-44BE-B049-B883-61DB3256096D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B89A541-A191-244D-AD62-E48D13259751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="41480" yWindow="-21100" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="wolfssl" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">wolfssl!$A$1:$V$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">wolfssl!$A$1:$X$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="119">
   <si>
     <t>Version</t>
   </si>
@@ -375,6 +375,15 @@
   </si>
   <si>
     <t>Empty/Incomplete Files</t>
+  </si>
+  <si>
+    <t>Clang_ministral</t>
+  </si>
+  <si>
+    <t>Clang_qwen3</t>
+  </si>
+  <si>
+    <t>Fail</t>
   </si>
 </sst>
 </file>
@@ -773,7 +782,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:W23"/>
+  <dimension ref="A1:Y23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -789,7 +798,7 @@
     <col min="12" max="12" width="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="14" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:25" s="14" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -839,26 +848,32 @@
         <v>10</v>
       </c>
       <c r="Q1" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="R1" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="S1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="T1" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="S1" s="8" t="s">
+      <c r="U1" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="V1" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="U1" s="8" t="s">
+      <c r="W1" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="V1" s="8" t="s">
+      <c r="X1" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="W1"/>
+      <c r="Y1"/>
     </row>
-    <row r="2" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:25" ht="15" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>44</v>
       </c>
@@ -902,23 +917,25 @@
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
-      <c r="R2" s="6" t="s">
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="S2">
-        <v>19939</v>
-      </c>
-      <c r="T2">
-        <v>20150</v>
       </c>
       <c r="U2">
         <v>19939</v>
       </c>
       <c r="V2">
+        <v>20150</v>
+      </c>
+      <c r="W2">
+        <v>19939</v>
+      </c>
+      <c r="X2">
         <v>20142</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:25" ht="15" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>51</v>
       </c>
@@ -964,11 +981,13 @@
         <v>82</v>
       </c>
       <c r="Q3" s="1"/>
-      <c r="R3" s="6" t="s">
+      <c r="R3" s="1"/>
+      <c r="S3" s="1"/>
+      <c r="T3" s="6" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:25" ht="15" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>51</v>
       </c>
@@ -1014,17 +1033,19 @@
         <v>82</v>
       </c>
       <c r="Q4" s="1"/>
-      <c r="R4" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="U4">
+      <c r="R4" s="1"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="W4">
         <v>11864</v>
       </c>
-      <c r="V4">
+      <c r="X4">
         <v>12272</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:25" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>26</v>
       </c>
@@ -1073,12 +1094,16 @@
       <c r="P5" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="Q5" s="1"/>
-      <c r="R5" s="6" t="s">
+      <c r="Q5" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="R5" s="1"/>
+      <c r="S5" s="1"/>
+      <c r="T5" s="6" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:25" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>26</v>
       </c>
@@ -1124,23 +1149,25 @@
         <v>82</v>
       </c>
       <c r="Q6" s="1"/>
-      <c r="R6" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="S6">
-        <v>8782</v>
-      </c>
-      <c r="T6">
-        <v>9606</v>
+      <c r="R6" s="1"/>
+      <c r="S6" s="1"/>
+      <c r="T6" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="U6">
         <v>8782</v>
       </c>
       <c r="V6">
+        <v>9606</v>
+      </c>
+      <c r="W6">
+        <v>8782</v>
+      </c>
+      <c r="X6">
         <v>9598</v>
       </c>
     </row>
-    <row r="7" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:25" ht="15" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -1189,18 +1216,22 @@
       <c r="P7" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="Q7" s="1"/>
-      <c r="R7" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="U7">
+      <c r="Q7" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="R7" s="1"/>
+      <c r="S7" s="1"/>
+      <c r="T7" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="W7">
         <v>993</v>
       </c>
-      <c r="V7">
+      <c r="X7">
         <v>1156</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:25" ht="15" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>12</v>
       </c>
@@ -1249,24 +1280,28 @@
       <c r="P8" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="Q8" s="1"/>
-      <c r="R8" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="S8">
+      <c r="Q8" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="R8" s="1"/>
+      <c r="S8" s="1"/>
+      <c r="T8" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="U8">
         <v>1692</v>
       </c>
-      <c r="T8">
+      <c r="V8">
         <v>1813</v>
       </c>
-      <c r="U8">
+      <c r="W8">
         <v>1797</v>
       </c>
-      <c r="V8">
+      <c r="X8">
         <v>1914</v>
       </c>
     </row>
-    <row r="9" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:25" ht="15" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
@@ -1312,23 +1347,25 @@
         <v>82</v>
       </c>
       <c r="Q9" s="1"/>
-      <c r="R9" s="6" t="s">
+      <c r="R9" s="1"/>
+      <c r="S9" s="1"/>
+      <c r="T9" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="S9">
+      <c r="U9">
         <v>2481</v>
       </c>
-      <c r="T9">
+      <c r="V9">
         <v>2660</v>
       </c>
-      <c r="U9">
+      <c r="W9">
         <v>2516</v>
       </c>
-      <c r="V9">
+      <c r="X9">
         <v>2695</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:25" ht="15" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>26</v>
       </c>
@@ -1372,23 +1409,25 @@
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
-      <c r="R10" s="6" t="s">
+      <c r="R10" s="1"/>
+      <c r="S10" s="1"/>
+      <c r="T10" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="S10">
+      <c r="U10">
         <v>654</v>
       </c>
-      <c r="T10">
+      <c r="V10">
         <v>686</v>
       </c>
-      <c r="U10">
+      <c r="W10">
         <v>653</v>
       </c>
-      <c r="V10">
+      <c r="X10">
         <v>685</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:25" ht="15" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>44</v>
       </c>
@@ -1438,14 +1477,10 @@
         <v>82</v>
       </c>
       <c r="Q11" s="1"/>
-      <c r="R11" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="S11">
-        <v>346</v>
-      </c>
-      <c r="T11">
-        <v>583</v>
+      <c r="R11" s="1"/>
+      <c r="S11" s="1"/>
+      <c r="T11" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="U11">
         <v>346</v>
@@ -1453,8 +1488,14 @@
       <c r="V11">
         <v>583</v>
       </c>
+      <c r="W11">
+        <v>346</v>
+      </c>
+      <c r="X11">
+        <v>583</v>
+      </c>
     </row>
-    <row r="12" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:25" ht="15" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>26</v>
       </c>
@@ -1495,14 +1536,16 @@
         <v>115</v>
       </c>
       <c r="P12" s="1"/>
-      <c r="Q12" s="1" t="s">
+      <c r="Q12" s="1"/>
+      <c r="R12" s="1"/>
+      <c r="S12" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="R12" s="6" t="s">
+      <c r="T12" s="6" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>40</v>
       </c>
@@ -1548,23 +1591,25 @@
         <v>82</v>
       </c>
       <c r="Q13" s="1"/>
-      <c r="R13" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="S13">
+      <c r="R13" s="1"/>
+      <c r="S13" s="1"/>
+      <c r="T13" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="U13">
         <v>20913</v>
       </c>
-      <c r="T13">
+      <c r="V13">
         <v>21203</v>
       </c>
-      <c r="U13">
+      <c r="W13">
         <v>20905</v>
       </c>
-      <c r="V13">
+      <c r="X13">
         <v>21195</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:25" ht="15" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>51</v>
       </c>
@@ -1610,23 +1655,25 @@
         <v>82</v>
       </c>
       <c r="Q14" s="1"/>
-      <c r="R14" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="S14">
-        <v>1030</v>
-      </c>
-      <c r="T14">
-        <v>1187</v>
+      <c r="R14" s="1"/>
+      <c r="S14" s="1"/>
+      <c r="T14" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="U14">
         <v>1030</v>
       </c>
       <c r="V14">
+        <v>1187</v>
+      </c>
+      <c r="W14">
+        <v>1030</v>
+      </c>
+      <c r="X14">
         <v>1184</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:25" ht="15" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>26</v>
       </c>
@@ -1670,23 +1717,25 @@
       <c r="O15" s="1"/>
       <c r="P15" s="1"/>
       <c r="Q15" s="1"/>
-      <c r="R15" s="6" t="s">
+      <c r="R15" s="1"/>
+      <c r="S15" s="1"/>
+      <c r="T15" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="S15">
-        <v>12845</v>
-      </c>
-      <c r="T15">
-        <v>13109</v>
       </c>
       <c r="U15">
         <v>12845</v>
       </c>
       <c r="V15">
+        <v>13109</v>
+      </c>
+      <c r="W15">
+        <v>12845</v>
+      </c>
+      <c r="X15">
         <v>13253</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:25" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>12</v>
       </c>
@@ -1735,18 +1784,22 @@
       <c r="P16" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="Q16" s="1"/>
-      <c r="R16" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="U16">
+      <c r="Q16" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="R16" s="1"/>
+      <c r="S16" s="1"/>
+      <c r="T16" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="W16">
         <v>1</v>
       </c>
-      <c r="V16">
+      <c r="X16">
         <v>164</v>
       </c>
     </row>
-    <row r="17" spans="1:22" ht="15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:24" ht="15" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>51</v>
       </c>
@@ -1792,14 +1845,10 @@
         <v>82</v>
       </c>
       <c r="Q17" s="1"/>
-      <c r="R17" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="S17">
-        <v>14423</v>
-      </c>
-      <c r="T17">
-        <v>14564</v>
+      <c r="R17" s="1"/>
+      <c r="S17" s="1"/>
+      <c r="T17" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="U17">
         <v>14423</v>
@@ -1807,8 +1856,14 @@
       <c r="V17">
         <v>14564</v>
       </c>
+      <c r="W17">
+        <v>14423</v>
+      </c>
+      <c r="X17">
+        <v>14564</v>
+      </c>
     </row>
-    <row r="18" spans="1:22" ht="15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:24" ht="15" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>26</v>
       </c>
@@ -1854,23 +1909,25 @@
         <v>82</v>
       </c>
       <c r="Q18" s="1"/>
-      <c r="R18" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="S18">
+      <c r="R18" s="1"/>
+      <c r="S18" s="1"/>
+      <c r="T18" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="U18">
         <v>38033</v>
       </c>
-      <c r="T18">
+      <c r="V18">
         <v>38113</v>
       </c>
-      <c r="U18">
+      <c r="W18">
         <v>38034</v>
       </c>
-      <c r="V18">
+      <c r="X18">
         <v>38111</v>
       </c>
     </row>
-    <row r="19" spans="1:22" ht="15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:24" ht="15" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>40</v>
       </c>
@@ -1913,12 +1970,16 @@
       <c r="P19" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="Q19" s="1"/>
-      <c r="R19" s="6" t="s">
+      <c r="Q19" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="R19" s="1"/>
+      <c r="S19" s="1"/>
+      <c r="T19" s="6" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="20" spans="1:22" ht="15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:24" ht="15" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>44</v>
       </c>
@@ -1964,23 +2025,25 @@
         <v>82</v>
       </c>
       <c r="Q20" s="1"/>
-      <c r="R20" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="S20">
+      <c r="R20" s="1"/>
+      <c r="S20" s="1"/>
+      <c r="T20" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="U20">
         <v>6437</v>
       </c>
-      <c r="T20">
+      <c r="V20">
         <v>6504</v>
       </c>
-      <c r="U20">
+      <c r="W20">
         <v>6443</v>
       </c>
-      <c r="V20">
+      <c r="X20">
         <v>6513</v>
       </c>
     </row>
-    <row r="21" spans="1:22" ht="15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:24" ht="15" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>26</v>
       </c>
@@ -2024,23 +2087,25 @@
       <c r="O21" s="1"/>
       <c r="P21" s="1"/>
       <c r="Q21" s="1"/>
-      <c r="R21" s="6" t="s">
+      <c r="R21" s="1"/>
+      <c r="S21" s="1"/>
+      <c r="T21" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="S21">
+      <c r="U21">
         <v>20966</v>
       </c>
-      <c r="T21">
+      <c r="V21">
         <v>21004</v>
       </c>
-      <c r="U21">
+      <c r="W21">
         <v>20965</v>
       </c>
-      <c r="V21">
+      <c r="X21">
         <v>21003</v>
       </c>
     </row>
-    <row r="22" spans="1:22" ht="15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:24" ht="15" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>12</v>
       </c>
@@ -2089,24 +2154,30 @@
       <c r="P22" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="Q22" s="1"/>
-      <c r="R22" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="S22">
+      <c r="Q22" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="R22" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="S22" s="1"/>
+      <c r="T22" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="U22">
         <v>6</v>
       </c>
-      <c r="T22">
+      <c r="V22">
         <v>119</v>
       </c>
-      <c r="U22">
+      <c r="W22">
         <v>69</v>
       </c>
-      <c r="V22">
+      <c r="X22">
         <v>185</v>
       </c>
     </row>
-    <row r="23" spans="1:22" ht="15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:24" ht="15" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>12</v>
       </c>
@@ -2155,25 +2226,31 @@
       <c r="P23" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="Q23" s="1"/>
-      <c r="R23" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="S23">
+      <c r="Q23" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="R23" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="S23" s="1"/>
+      <c r="T23" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="U23">
         <v>325</v>
       </c>
-      <c r="T23">
+      <c r="V23">
         <v>419</v>
       </c>
-      <c r="U23">
+      <c r="W23">
         <v>323</v>
       </c>
-      <c r="V23">
+      <c r="X23">
         <v>417</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:X1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>